<commit_message>
Updated sections Purpose, Exec Summary, Project Description, scope and business drivers following Workshop 2 and Email
</commit_message>
<xml_diff>
--- a/docs/project-management/02_Business_Requirements/BRD-Review-Log-v0.1.xlsx
+++ b/docs/project-management/02_Business_Requirements/BRD-Review-Log-v0.1.xlsx
@@ -5,26 +5,27 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d752cb73b61fc091/Desktop/linuxlabs/projectredstone/docs/project-management/01_Discovery/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d752cb73b61fc091/Desktop/linuxlabs/projectredstone/docs/project-management/02_Business_Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="182" documentId="8_{A8AD7E28-50AD-41CA-B798-B213AEC76627}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE786EC1-BD4F-4829-99FA-E18E38D0A215}"/>
+  <xr:revisionPtr revIDLastSave="198" documentId="8_{A8AD7E28-50AD-41CA-B798-B213AEC76627}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{81CAF48C-042A-4EF6-BDF5-797DAC386BD3}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{76AF004E-0D5E-43C6-8E8F-EE458AB65108}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{76AF004E-0D5E-43C6-8E8F-EE458AB65108}"/>
   </bookViews>
   <sheets>
     <sheet name="Workshop 2 Actions Log" sheetId="7" r:id="rId1"/>
-    <sheet name="BRD CRs" sheetId="1" r:id="rId2"/>
-    <sheet name="Decision Points" sheetId="2" r:id="rId3"/>
-    <sheet name="CR-001" sheetId="3" r:id="rId4"/>
-    <sheet name="CR-004" sheetId="4" r:id="rId5"/>
-    <sheet name="CR-005" sheetId="5" r:id="rId6"/>
-    <sheet name="CR-006" sheetId="6" r:id="rId7"/>
-    <sheet name="CR-007" sheetId="8" r:id="rId8"/>
-    <sheet name="CR-009" sheetId="9" r:id="rId9"/>
-    <sheet name="CR-010" sheetId="10" r:id="rId10"/>
-    <sheet name="CR-011" sheetId="11" r:id="rId11"/>
-    <sheet name="DP-015" sheetId="12" r:id="rId12"/>
+    <sheet name="Sheet1" sheetId="13" r:id="rId2"/>
+    <sheet name="BRD CRs" sheetId="1" r:id="rId3"/>
+    <sheet name="Decision Points" sheetId="2" r:id="rId4"/>
+    <sheet name="CR-001" sheetId="3" r:id="rId5"/>
+    <sheet name="CR-004" sheetId="4" r:id="rId6"/>
+    <sheet name="CR-005" sheetId="5" r:id="rId7"/>
+    <sheet name="CR-006" sheetId="6" r:id="rId8"/>
+    <sheet name="CR-007" sheetId="8" r:id="rId9"/>
+    <sheet name="CR-009" sheetId="9" r:id="rId10"/>
+    <sheet name="CR-010" sheetId="10" r:id="rId11"/>
+    <sheet name="CR-011" sheetId="11" r:id="rId12"/>
+    <sheet name="DP-015" sheetId="12" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -50,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="697" uniqueCount="550">
   <si>
     <t>Ref</t>
   </si>
@@ -1082,6 +1083,670 @@
   </si>
   <si>
     <t>After approval</t>
+  </si>
+  <si>
+    <t>Section / Area</t>
+  </si>
+  <si>
+    <t>Workshop 2 change</t>
+  </si>
+  <si>
+    <t>Sarah's email / RHCSA coverage change</t>
+  </si>
+  <si>
+    <t>v1.0 action</t>
+  </si>
+  <si>
+    <t>Document Control</t>
+  </si>
+  <si>
+    <t>BRD approved for baseline after updates</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Change version to </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1.0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, update date and revision history</t>
+    </r>
+  </si>
+  <si>
+    <t>1. Purpose</t>
+  </si>
+  <si>
+    <t>BRD now represents completed requirements gathering</t>
+  </si>
+  <si>
+    <t>Clarify that v1.0 establishes the baseline for design</t>
+  </si>
+  <si>
+    <t>2. Executive Summary</t>
+  </si>
+  <si>
+    <t>Reflect Workshop 2 outcomes</t>
+  </si>
+  <si>
+    <t>Reflect expanded operational capabilities</t>
+  </si>
+  <si>
+    <t>Rewrite executive summary</t>
+  </si>
+  <si>
+    <t>3. Project Description</t>
+  </si>
+  <si>
+    <t>Incorporate refined requirements</t>
+  </si>
+  <si>
+    <t>Include improved administration, automation, recovery and operational maturity</t>
+  </si>
+  <si>
+    <t>Update</t>
+  </si>
+  <si>
+    <t>4. Scope</t>
+  </si>
+  <si>
+    <t>Documentation, asset management, testing and operational processes clarified</t>
+  </si>
+  <si>
+    <t>Automation, software management, recovery and operational administration</t>
+  </si>
+  <si>
+    <t>Expand scope where appropriate</t>
+  </si>
+  <si>
+    <t>5. Business Drivers</t>
+  </si>
+  <si>
+    <t>Growth assumptions updated</t>
+  </si>
+  <si>
+    <t>Operational efficiency strengthened through automation/standardisation</t>
+  </si>
+  <si>
+    <t>Review/update</t>
+  </si>
+  <si>
+    <t>6. Current State</t>
+  </si>
+  <si>
+    <t>Asset baseline remains outstanding</t>
+  </si>
+  <si>
+    <t>Record current information without inventing asset figures</t>
+  </si>
+  <si>
+    <t>7. Delivery Approach</t>
+  </si>
+  <si>
+    <t>Controlled migration, UAT and pre-production testing discussed</t>
+  </si>
+  <si>
+    <t>Software/update testing reinforced</t>
+  </si>
+  <si>
+    <t>Update delivery/testing language</t>
+  </si>
+  <si>
+    <t>7. Governance</t>
+  </si>
+  <si>
+    <t>Formal RTM, change management and acceptance</t>
+  </si>
+  <si>
+    <t>Retain, refine where necessary</t>
+  </si>
+  <si>
+    <t>BR-001 Business Service Continuity</t>
+  </si>
+  <si>
+    <t>Clarify continuity expectations</t>
+  </si>
+  <si>
+    <t>Recovery requirements reinforced</t>
+  </si>
+  <si>
+    <t>Review acceptance criteria</t>
+  </si>
+  <si>
+    <t>BR-002 Identity Management</t>
+  </si>
+  <si>
+    <t>HR/IT ownership discussed</t>
+  </si>
+  <si>
+    <t>Refine ownership/process language</t>
+  </si>
+  <si>
+    <t>BR-003 User Provisioning</t>
+  </si>
+  <si>
+    <t>Joiner/mover/leaver process</t>
+  </si>
+  <si>
+    <t>Automation of repetitive administration</t>
+  </si>
+  <si>
+    <t>Expand into controlled lifecycle + automation</t>
+  </si>
+  <si>
+    <t>BR-004 RBAC</t>
+  </si>
+  <si>
+    <t>Host/resource security reinforced</t>
+  </si>
+  <si>
+    <t>Review relationship with security requirements</t>
+  </si>
+  <si>
+    <t>BR-005 File Services</t>
+  </si>
+  <si>
+    <t>Network resource access</t>
+  </si>
+  <si>
+    <t>Ensure network-based resource access is explicitly covered</t>
+  </si>
+  <si>
+    <t>BR-006 Data Organisation</t>
+  </si>
+  <si>
+    <t>Naming conventions</t>
+  </si>
+  <si>
+    <t>Retain/update</t>
+  </si>
+  <si>
+    <t>BR-007 Data Segregation</t>
+  </si>
+  <si>
+    <t>Security enforcement</t>
+  </si>
+  <si>
+    <t>Review for host-level access controls</t>
+  </si>
+  <si>
+    <t>BR-008 Secure Data Access</t>
+  </si>
+  <si>
+    <t>Security enforcement/auditability</t>
+  </si>
+  <si>
+    <t>Strengthen where necessary</t>
+  </si>
+  <si>
+    <t>BR-009 Centralised Logging</t>
+  </si>
+  <si>
+    <t>Persistent operational logging</t>
+  </si>
+  <si>
+    <t>Expand requirement to cover log persistence/retention</t>
+  </si>
+  <si>
+    <t>BR-010 Monitoring</t>
+  </si>
+  <si>
+    <t>Split operational monitoring from capacity/performance management</t>
+  </si>
+  <si>
+    <t>Performance management reinforced</t>
+  </si>
+  <si>
+    <t>Split/expand requirement</t>
+  </si>
+  <si>
+    <t>New – Capacity &amp; Performance</t>
+  </si>
+  <si>
+    <t>Monthly capacity/performance reporting</t>
+  </si>
+  <si>
+    <t>Performance identification and remediation</t>
+  </si>
+  <si>
+    <t>Add new BR</t>
+  </si>
+  <si>
+    <t>BR-011 Threat Detection</t>
+  </si>
+  <si>
+    <t>Security controls</t>
+  </si>
+  <si>
+    <t>Review but don't over-specify technology</t>
+  </si>
+  <si>
+    <t>BR-012 Backups</t>
+  </si>
+  <si>
+    <t>Automated backups</t>
+  </si>
+  <si>
+    <t>Scheduled administration</t>
+  </si>
+  <si>
+    <t>Retain + strengthen scheduling</t>
+  </si>
+  <si>
+    <t>BR-013 Backup Validation</t>
+  </si>
+  <si>
+    <t>Recovery testing</t>
+  </si>
+  <si>
+    <t>System recovery</t>
+  </si>
+  <si>
+    <t>Expand recovery requirement</t>
+  </si>
+  <si>
+    <t>BR-014 Application Resilience</t>
+  </si>
+  <si>
+    <t>HA remains decision point</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Do </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>not</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> mandate HA; document as design decision</t>
+    </r>
+  </si>
+  <si>
+    <t>BR-015 Remote Administration</t>
+  </si>
+  <si>
+    <t>Administrative capabilities</t>
+  </si>
+  <si>
+    <t>Retain</t>
+  </si>
+  <si>
+    <t>BR-016 Secure Remote Access</t>
+  </si>
+  <si>
+    <t>Remote/office users should have consistent experience</t>
+  </si>
+  <si>
+    <t>Refine UX requirement</t>
+  </si>
+  <si>
+    <t>BR-017 Network Security</t>
+  </si>
+  <si>
+    <t>Firewall/internet access requirement</t>
+  </si>
+  <si>
+    <t>Host-level security</t>
+  </si>
+  <si>
+    <t>Review</t>
+  </si>
+  <si>
+    <t>BR-018 Network Segmentation</t>
+  </si>
+  <si>
+    <t>BR-019 Integration</t>
+  </si>
+  <si>
+    <t>Microsoft 365 / existing services</t>
+  </si>
+  <si>
+    <t>Review integration wording</t>
+  </si>
+  <si>
+    <t>BR-020 Application Hosting</t>
+  </si>
+  <si>
+    <t>BR-021 Scalability</t>
+  </si>
+  <si>
+    <t>Growth forecast updated</t>
+  </si>
+  <si>
+    <t>Update five-year assumptions</t>
+  </si>
+  <si>
+    <t>BR-022 Standardisation</t>
+  </si>
+  <si>
+    <t>Automation/controlled administration</t>
+  </si>
+  <si>
+    <t>Strengthen</t>
+  </si>
+  <si>
+    <t>BR-023 Documentation</t>
+  </si>
+  <si>
+    <t>SOPs + runbooks explicitly required</t>
+  </si>
+  <si>
+    <t>Recovery/troubleshooting procedures</t>
+  </si>
+  <si>
+    <t>Expand to distinguish SOPs, runbooks and user documentation</t>
+  </si>
+  <si>
+    <t>BR-024 Reporting</t>
+  </si>
+  <si>
+    <t>Operational vs management reporting clarified</t>
+  </si>
+  <si>
+    <t>Performance/capacity reporting</t>
+  </si>
+  <si>
+    <t>Refine</t>
+  </si>
+  <si>
+    <t>BR-025 Approval Workflows</t>
+  </si>
+  <si>
+    <t>Review; avoid unnecessary scope</t>
+  </si>
+  <si>
+    <t>BR-026 Print Services</t>
+  </si>
+  <si>
+    <t>Network printing requirement confirmed</t>
+  </si>
+  <si>
+    <t>New – Asset Management</t>
+  </si>
+  <si>
+    <t>Formal IT asset management introduced</t>
+  </si>
+  <si>
+    <t>Add BR</t>
+  </si>
+  <si>
+    <t>New – Software Update Management</t>
+  </si>
+  <si>
+    <t>Controlled update process + sandbox testing</t>
+  </si>
+  <si>
+    <t>Software/package lifecycle</t>
+  </si>
+  <si>
+    <t>New – Joiner/Mover/Leaver Process</t>
+  </si>
+  <si>
+    <t>Ownership/process clarification</t>
+  </si>
+  <si>
+    <t>Automation</t>
+  </si>
+  <si>
+    <t>Add or restructure BR-003</t>
+  </si>
+  <si>
+    <t>New – Administrative Automation</t>
+  </si>
+  <si>
+    <t>Explicit automation requirement</t>
+  </si>
+  <si>
+    <t>New – Scheduled Administration</t>
+  </si>
+  <si>
+    <t>Scheduling of routine tasks</t>
+  </si>
+  <si>
+    <t>Add BR or incorporate into operational management</t>
+  </si>
+  <si>
+    <t>New – System Recovery</t>
+  </si>
+  <si>
+    <t>RTO/RPO discussion</t>
+  </si>
+  <si>
+    <t>Boot/configuration/service recovery</t>
+  </si>
+  <si>
+    <t>New – Time Synchronisation</t>
+  </si>
+  <si>
+    <t>Consistent system time</t>
+  </si>
+  <si>
+    <t>New – Host Security Enforcement</t>
+  </si>
+  <si>
+    <t>Explicit security enforcement</t>
+  </si>
+  <si>
+    <t>Add/refine BR</t>
+  </si>
+  <si>
+    <t>New – Network Resource Mounting/Access</t>
+  </si>
+  <si>
+    <t>File services</t>
+  </si>
+  <si>
+    <t>Automated network resource access</t>
+  </si>
+  <si>
+    <t>Add if not sufficiently covered by file-services requirement</t>
+  </si>
+  <si>
+    <t>NFR-001 Availability</t>
+  </si>
+  <si>
+    <t>HA decision point</t>
+  </si>
+  <si>
+    <t>Clarify availability expectations without mandating HA</t>
+  </si>
+  <si>
+    <t>NFR-002 Reliability</t>
+  </si>
+  <si>
+    <t>Recovery/troubleshooting</t>
+  </si>
+  <si>
+    <t>NFR-003 Performance</t>
+  </si>
+  <si>
+    <t>Capacity/performance discussion</t>
+  </si>
+  <si>
+    <t>Performance management</t>
+  </si>
+  <si>
+    <t>NFR-004 Scalability</t>
+  </si>
+  <si>
+    <t>Growth updated</t>
+  </si>
+  <si>
+    <t>NFR-005 Security</t>
+  </si>
+  <si>
+    <t>Host-level security enforcement</t>
+  </si>
+  <si>
+    <t>NFR-006 Auditability</t>
+  </si>
+  <si>
+    <t>Persistent logs</t>
+  </si>
+  <si>
+    <t>NFR-007 Data Protection</t>
+  </si>
+  <si>
+    <t>NFR-008 Maintainability</t>
+  </si>
+  <si>
+    <t>Maintenance process</t>
+  </si>
+  <si>
+    <t>Automation/scheduling</t>
+  </si>
+  <si>
+    <t>NFR-009 Recoverability</t>
+  </si>
+  <si>
+    <t>4-hour expectation discussed</t>
+  </si>
+  <si>
+    <t>Major update</t>
+  </si>
+  <si>
+    <t>NFR-010 Supportability</t>
+  </si>
+  <si>
+    <t>SOPs/runbooks</t>
+  </si>
+  <si>
+    <t>Troubleshooting/recovery documentation</t>
+  </si>
+  <si>
+    <t>Expand</t>
+  </si>
+  <si>
+    <t>NFR-011 Administrative Simplicity</t>
+  </si>
+  <si>
+    <t>NFR-012 Compatibility</t>
+  </si>
+  <si>
+    <t>Existing applications</t>
+  </si>
+  <si>
+    <t>Software/update testing</t>
+  </si>
+  <si>
+    <t>NFR-013 Compliance</t>
+  </si>
+  <si>
+    <t>NFR-014 Monitoring</t>
+  </si>
+  <si>
+    <t>Operational monitoring split from capacity</t>
+  </si>
+  <si>
+    <t>NFR-015 Extensibility</t>
+  </si>
+  <si>
+    <t>Future growth</t>
+  </si>
+  <si>
+    <t>New NFR – Time Consistency</t>
+  </si>
+  <si>
+    <t>System time</t>
+  </si>
+  <si>
+    <t>Add if better expressed as NFR</t>
+  </si>
+  <si>
+    <t>New NFR – Recovery</t>
+  </si>
+  <si>
+    <t>4-hour business expectation</t>
+  </si>
+  <si>
+    <t>Recovery procedures</t>
+  </si>
+  <si>
+    <t>Add/strengthen as appropriate</t>
+  </si>
+  <si>
+    <t>Assumptions</t>
+  </si>
+  <si>
+    <t>Asset inventory, SMEs, growth information</t>
+  </si>
+  <si>
+    <t>Update outstanding dependencies</t>
+  </si>
+  <si>
+    <t>Constraints</t>
+  </si>
+  <si>
+    <t>Migration downtime</t>
+  </si>
+  <si>
+    <t>Add migration constraints</t>
+  </si>
+  <si>
+    <t>Risks</t>
+  </si>
+  <si>
+    <t>Migration, update testing, asset information</t>
+  </si>
+  <si>
+    <t>Expand risk register</t>
+  </si>
+  <si>
+    <t>Success Criteria</t>
+  </si>
+  <si>
+    <t>UAT, documentation, operational handover</t>
+  </si>
+  <si>
+    <t>Expanded operational capability</t>
+  </si>
+  <si>
+    <t>Appendix / Priority</t>
+  </si>
+  <si>
+    <t>MoSCoW confirmed</t>
+  </si>
+  <si>
+    <t>Review priority definitions for consistency</t>
+  </si>
+  <si>
+    <t>Complete</t>
+  </si>
+  <si>
+    <t>Y</t>
   </si>
 </sst>
 </file>
@@ -1591,6 +2256,49 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AC1AD7B-E970-4F09-A680-C6B19B85275B}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultColWidth="35" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>302</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>307</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91875EC5-C451-43C7-A93D-44CC0EDE49B4}">
   <dimension ref="A1:A3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1613,7 +2321,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0AAEABD2-DF3D-4BB6-BA28-24FD04925B8C}">
   <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1666,7 +2374,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{058578A8-981A-438B-97F6-53DFB1F765F4}">
   <dimension ref="A1:A16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1743,6 +2451,996 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{453F13AB-2197-416E-93CC-5F22120082A4}">
+  <dimension ref="A1:E68"/>
+  <sheetFormatPr defaultColWidth="94.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" customWidth="1"/>
+    <col min="2" max="2" width="40.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="73" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="73.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="57.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>548</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>549</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>549</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>549</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>549</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>549</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>363</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>549</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B8" s="6" t="s">
+        <v>371</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B9" s="6" t="s">
+        <v>374</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B10" s="6" t="s">
+        <v>378</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B11" s="6" t="s">
+        <v>381</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>382</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>383</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B12" s="6" t="s">
+        <v>385</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B13" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>389</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B14" s="6" t="s">
+        <v>392</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B15" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>396</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B16" s="6" t="s">
+        <v>398</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>399</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B17" s="6" t="s">
+        <v>401</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B18" s="6" t="s">
+        <v>404</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>405</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B19" s="6" t="s">
+        <v>407</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B20" s="6" t="s">
+        <v>410</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B21" s="6" t="s">
+        <v>414</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B22" s="6" t="s">
+        <v>418</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B23" s="6" t="s">
+        <v>421</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B24" s="6" t="s">
+        <v>425</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B25" s="6" t="s">
+        <v>429</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B26" s="6" t="s">
+        <v>432</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>433</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B27" s="6" t="s">
+        <v>435</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B28" s="6" t="s">
+        <v>438</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>440</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B29" s="6" t="s">
+        <v>442</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B30" s="6" t="s">
+        <v>443</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B31" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B32" s="6" t="s">
+        <v>447</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>448</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B33" s="6" t="s">
+        <v>450</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B34" s="6" t="s">
+        <v>453</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>455</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B35" s="6" t="s">
+        <v>457</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>458</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>459</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B36" s="6" t="s">
+        <v>461</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="37" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B37" s="6" t="s">
+        <v>463</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>464</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="38" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B38" s="6" t="s">
+        <v>465</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>466</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="39" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B39" s="6" t="s">
+        <v>468</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>469</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>470</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="40" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B40" s="6" t="s">
+        <v>471</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>472</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>473</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="41" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B41" s="6" t="s">
+        <v>475</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>476</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="42" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B42" s="6" t="s">
+        <v>477</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>478</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="43" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B43" s="6" t="s">
+        <v>480</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>481</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="44" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B44" s="6" t="s">
+        <v>483</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="45" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B45" s="6" t="s">
+        <v>485</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="46" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B46" s="6" t="s">
+        <v>488</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>489</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="47" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B47" s="6" t="s">
+        <v>492</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>493</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="48" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B48" s="6" t="s">
+        <v>495</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="49" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B49" s="6" t="s">
+        <v>497</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="50" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B50" s="6" t="s">
+        <v>500</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>501</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="51" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B51" s="6" t="s">
+        <v>502</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="52" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B52" s="6" t="s">
+        <v>504</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>505</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="53" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B53" s="6" t="s">
+        <v>506</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="54" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B54" s="6" t="s">
+        <v>507</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>508</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>509</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="55" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B55" s="6" t="s">
+        <v>510</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>511</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="E55" s="6" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="56" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B56" s="6" t="s">
+        <v>513</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>514</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="57" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B57" s="6" t="s">
+        <v>517</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>473</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="58" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B58" s="6" t="s">
+        <v>518</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="59" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B59" s="6" t="s">
+        <v>521</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="60" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B60" s="6" t="s">
+        <v>522</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="61" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B61" s="6" t="s">
+        <v>524</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="62" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B62" s="6" t="s">
+        <v>526</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>527</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="63" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B63" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>530</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>531</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="64" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B64" s="6" t="s">
+        <v>533</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="65" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B65" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>537</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="66" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B66" s="6" t="s">
+        <v>539</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>540</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="67" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B67" s="6" t="s">
+        <v>542</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>543</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>544</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="68" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B68" s="6" t="s">
+        <v>545</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>546</v>
+      </c>
+      <c r="D68" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>547</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40E84F65-51B6-44B5-90F8-5E4AD20D77E4}">
   <dimension ref="A1:G13"/>
   <sheetFormatPr defaultColWidth="40.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2058,7 +3756,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92C32BAD-19BD-430E-85DE-E32588222CF6}">
   <dimension ref="A1:E26"/>
   <sheetFormatPr defaultColWidth="40.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2516,7 +4214,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{760DEA66-EF41-4777-8D42-2FC12487128B}">
   <dimension ref="A1:F13"/>
   <sheetFormatPr defaultColWidth="57.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2698,7 +4396,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{119F2194-0B3D-4FAD-BA62-27A84560F9AA}">
   <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="32.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2811,7 +4509,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42010116-26CA-4BA4-9B8D-EE715FFB1F5A}">
   <dimension ref="A1:C22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2972,7 +4670,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73D9C91B-B0AC-43D9-A2D4-AFEB03B2A6D4}">
   <dimension ref="A1:A18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3055,7 +4753,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A79D85F-4140-4F1C-BC56-63DB1809BF07}">
   <dimension ref="A1:A21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3154,47 +4852,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AC1AD7B-E970-4F09-A680-C6B19B85275B}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultColWidth="35" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>299</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>300</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>302</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
-        <v>305</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>307</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>